<commit_message>
Revisión documentacion inicial: 20-05-2026
</commit_message>
<xml_diff>
--- a/docs/04-evolutivo/Inventario_Deuda_Tecnica_v2.xlsx
+++ b/docs/04-evolutivo/Inventario_Deuda_Tecnica_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josegalinde/code/github/f5-proyecto-abandono-escolar/docs/04-evolutivo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED923D7-5462-644A-9A26-B3ECB2481446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F539B7E-4AEE-9E4E-A3C0-7692A816277F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17120" yWindow="2260" windowWidth="14180" windowHeight="17180" activeTab="2" xr2:uid="{A8A8EE6C-32F2-BE4A-B073-0068AE54B322}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="228">
   <si>
     <t>INVENTARIO DE DEUDA TECNICA INTERNA</t>
   </si>
@@ -2358,11 +2358,23 @@
       <c r="B71" s="3" t="s">
         <v>212</v>
       </c>
+      <c r="C71" t="s">
+        <v>221</v>
+      </c>
+      <c r="D71" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="72" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B72" s="3" t="s">
         <v>213</v>
       </c>
+      <c r="C72" t="s">
+        <v>225</v>
+      </c>
+      <c r="D72" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="73" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B73" s="3" t="s">
@@ -2391,28 +2403,46 @@
       <c r="C77" t="s">
         <v>221</v>
       </c>
+      <c r="D77" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="78" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B78" s="3" t="s">
         <v>217</v>
       </c>
+      <c r="C78" t="s">
+        <v>225</v>
+      </c>
+      <c r="D78" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="79" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B79" s="3" t="s">
         <v>218</v>
       </c>
+      <c r="C79" t="s">
+        <v>225</v>
+      </c>
+      <c r="D79" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="80" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B80" s="3" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="81" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="81" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B81" s="3" t="s">
         <v>219</v>
       </c>
       <c r="C81" t="s">
         <v>221</v>
+      </c>
+      <c r="D81" t="s">
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revisión documentacion inicial(revisión): 20-05-2026
</commit_message>
<xml_diff>
--- a/docs/04-evolutivo/Inventario_Deuda_Tecnica_v2.xlsx
+++ b/docs/04-evolutivo/Inventario_Deuda_Tecnica_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josegalinde/code/github/f5-proyecto-abandono-escolar/docs/04-evolutivo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F539B7E-4AEE-9E4E-A3C0-7692A816277F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA07C548-C166-9C4F-B254-09699FDDDB5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17120" yWindow="2260" windowWidth="14180" windowHeight="17180" activeTab="2" xr2:uid="{A8A8EE6C-32F2-BE4A-B073-0068AE54B322}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="228">
   <si>
     <t>INVENTARIO DE DEUDA TECNICA INTERNA</t>
   </si>
@@ -2058,6 +2058,9 @@
       <c r="B23" s="3" t="s">
         <v>182</v>
       </c>
+      <c r="C23" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B24" s="3" t="s">

</xml_diff>